<commit_message>
Update project Gantt chart
Updated the project Gantt diagram document to reflect revised scheduling details. This change keeps the Excel timeline aligned with the latest project planning information.
</commit_message>
<xml_diff>
--- a/Doc/Diagrama Gantt-Coluccio,V - Gomez, F.xlsx
+++ b/Doc/Diagrama Gantt-Coluccio,V - Gomez, F.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f3364099f710d5d8/Mis cosas/Facu/GitHub/Almacenamiento-con-Grua-Torre-Coluccio-Gomez/Doc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1475" documentId="8_{96292F3E-0F34-40E0-BFDE-1992214EE5CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE134E00-846F-4999-86F8-9E8F48687F1B}"/>
+  <xr:revisionPtr revIDLastSave="1476" documentId="8_{96292F3E-0F34-40E0-BFDE-1992214EE5CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{25268937-E92C-4161-987C-9EC03A670F36}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{78FD6F9D-33A7-4792-8E36-2E2F0DF50943}"/>
   </bookViews>
@@ -670,7 +670,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -866,69 +866,62 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1368,42 +1361,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:102" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="72" t="s">
+      <c r="A1" s="83" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
-      <c r="F1" s="72"/>
-      <c r="G1" s="72"/>
-      <c r="H1" s="72"/>
-      <c r="I1" s="72"/>
-      <c r="J1" s="72"/>
+      <c r="B1" s="83"/>
+      <c r="C1" s="83"/>
+      <c r="D1" s="83"/>
+      <c r="E1" s="83"/>
+      <c r="F1" s="83"/>
+      <c r="G1" s="83"/>
+      <c r="H1" s="83"/>
+      <c r="I1" s="83"/>
+      <c r="J1" s="83"/>
     </row>
     <row r="2" spans="1:102" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="72"/>
-      <c r="B2" s="72"/>
-      <c r="C2" s="72"/>
-      <c r="D2" s="72"/>
-      <c r="E2" s="72"/>
-      <c r="F2" s="72"/>
-      <c r="G2" s="72"/>
-      <c r="H2" s="72"/>
-      <c r="I2" s="72"/>
-      <c r="J2" s="72"/>
+      <c r="A2" s="83"/>
+      <c r="B2" s="83"/>
+      <c r="C2" s="83"/>
+      <c r="D2" s="83"/>
+      <c r="E2" s="83"/>
+      <c r="F2" s="83"/>
+      <c r="G2" s="83"/>
+      <c r="H2" s="83"/>
+      <c r="I2" s="83"/>
+      <c r="J2" s="83"/>
     </row>
     <row r="3" spans="1:102" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="72"/>
-      <c r="B3" s="72"/>
-      <c r="C3" s="72"/>
-      <c r="D3" s="72"/>
-      <c r="E3" s="72"/>
-      <c r="F3" s="72"/>
-      <c r="G3" s="72"/>
-      <c r="H3" s="72"/>
-      <c r="I3" s="72"/>
-      <c r="J3" s="72"/>
+      <c r="A3" s="83"/>
+      <c r="B3" s="83"/>
+      <c r="C3" s="83"/>
+      <c r="D3" s="83"/>
+      <c r="E3" s="83"/>
+      <c r="F3" s="83"/>
+      <c r="G3" s="83"/>
+      <c r="H3" s="83"/>
+      <c r="I3" s="83"/>
+      <c r="J3" s="83"/>
     </row>
     <row r="4" spans="1:102" s="19" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="17" t="s">
@@ -1424,136 +1417,136 @@
       <c r="I4" s="44"/>
       <c r="J4" s="17"/>
       <c r="K4" s="15"/>
-      <c r="L4" s="74">
+      <c r="L4" s="85">
         <f>L5</f>
         <v>45754</v>
       </c>
-      <c r="M4" s="70"/>
-      <c r="N4" s="70"/>
-      <c r="O4" s="70"/>
-      <c r="P4" s="70"/>
-      <c r="Q4" s="70"/>
-      <c r="R4" s="70"/>
-      <c r="S4" s="69">
+      <c r="M4" s="82"/>
+      <c r="N4" s="82"/>
+      <c r="O4" s="82"/>
+      <c r="P4" s="82"/>
+      <c r="Q4" s="82"/>
+      <c r="R4" s="82"/>
+      <c r="S4" s="86">
         <f t="shared" ref="S4" si="0">S5</f>
         <v>45761</v>
       </c>
-      <c r="T4" s="70"/>
-      <c r="U4" s="70"/>
-      <c r="V4" s="70"/>
-      <c r="W4" s="70"/>
-      <c r="X4" s="70"/>
-      <c r="Y4" s="71"/>
-      <c r="Z4" s="69">
+      <c r="T4" s="82"/>
+      <c r="U4" s="82"/>
+      <c r="V4" s="82"/>
+      <c r="W4" s="82"/>
+      <c r="X4" s="82"/>
+      <c r="Y4" s="87"/>
+      <c r="Z4" s="86">
         <f t="shared" ref="Z4" si="1">Z5</f>
         <v>45768</v>
       </c>
-      <c r="AA4" s="70"/>
-      <c r="AB4" s="70"/>
-      <c r="AC4" s="70"/>
-      <c r="AD4" s="70"/>
-      <c r="AE4" s="70"/>
-      <c r="AF4" s="71"/>
-      <c r="AG4" s="69">
+      <c r="AA4" s="82"/>
+      <c r="AB4" s="82"/>
+      <c r="AC4" s="82"/>
+      <c r="AD4" s="82"/>
+      <c r="AE4" s="82"/>
+      <c r="AF4" s="87"/>
+      <c r="AG4" s="86">
         <f t="shared" ref="AG4" si="2">AG5</f>
         <v>45775</v>
       </c>
-      <c r="AH4" s="70"/>
-      <c r="AI4" s="70"/>
-      <c r="AJ4" s="70"/>
-      <c r="AK4" s="70"/>
-      <c r="AL4" s="70"/>
-      <c r="AM4" s="71"/>
-      <c r="AN4" s="70">
+      <c r="AH4" s="82"/>
+      <c r="AI4" s="82"/>
+      <c r="AJ4" s="82"/>
+      <c r="AK4" s="82"/>
+      <c r="AL4" s="82"/>
+      <c r="AM4" s="87"/>
+      <c r="AN4" s="82">
         <f t="shared" ref="AN4" si="3">AN5</f>
         <v>45782</v>
       </c>
-      <c r="AO4" s="70"/>
-      <c r="AP4" s="70"/>
-      <c r="AQ4" s="70"/>
-      <c r="AR4" s="70"/>
-      <c r="AS4" s="70"/>
-      <c r="AT4" s="70"/>
-      <c r="AU4" s="69">
+      <c r="AO4" s="82"/>
+      <c r="AP4" s="82"/>
+      <c r="AQ4" s="82"/>
+      <c r="AR4" s="82"/>
+      <c r="AS4" s="82"/>
+      <c r="AT4" s="82"/>
+      <c r="AU4" s="86">
         <f t="shared" ref="AU4" si="4">AU5</f>
         <v>45789</v>
       </c>
-      <c r="AV4" s="70"/>
-      <c r="AW4" s="70"/>
-      <c r="AX4" s="70"/>
-      <c r="AY4" s="70"/>
-      <c r="AZ4" s="70"/>
-      <c r="BA4" s="71"/>
-      <c r="BB4" s="69">
+      <c r="AV4" s="82"/>
+      <c r="AW4" s="82"/>
+      <c r="AX4" s="82"/>
+      <c r="AY4" s="82"/>
+      <c r="AZ4" s="82"/>
+      <c r="BA4" s="87"/>
+      <c r="BB4" s="86">
         <f t="shared" ref="BB4" si="5">BB5</f>
         <v>45796</v>
       </c>
-      <c r="BC4" s="70"/>
-      <c r="BD4" s="70"/>
-      <c r="BE4" s="70"/>
-      <c r="BF4" s="70"/>
-      <c r="BG4" s="70"/>
-      <c r="BH4" s="71"/>
-      <c r="BI4" s="69">
+      <c r="BC4" s="82"/>
+      <c r="BD4" s="82"/>
+      <c r="BE4" s="82"/>
+      <c r="BF4" s="82"/>
+      <c r="BG4" s="82"/>
+      <c r="BH4" s="87"/>
+      <c r="BI4" s="86">
         <f t="shared" ref="BI4" si="6">BI5</f>
         <v>45803</v>
       </c>
-      <c r="BJ4" s="70"/>
-      <c r="BK4" s="70"/>
-      <c r="BL4" s="70"/>
-      <c r="BM4" s="70"/>
-      <c r="BN4" s="70"/>
-      <c r="BO4" s="71"/>
-      <c r="BP4" s="69">
+      <c r="BJ4" s="82"/>
+      <c r="BK4" s="82"/>
+      <c r="BL4" s="82"/>
+      <c r="BM4" s="82"/>
+      <c r="BN4" s="82"/>
+      <c r="BO4" s="87"/>
+      <c r="BP4" s="86">
         <f t="shared" ref="BP4" si="7">BP5</f>
         <v>45810</v>
       </c>
-      <c r="BQ4" s="70"/>
-      <c r="BR4" s="70"/>
-      <c r="BS4" s="70"/>
-      <c r="BT4" s="70"/>
-      <c r="BU4" s="70"/>
-      <c r="BV4" s="71"/>
-      <c r="BW4" s="69">
+      <c r="BQ4" s="82"/>
+      <c r="BR4" s="82"/>
+      <c r="BS4" s="82"/>
+      <c r="BT4" s="82"/>
+      <c r="BU4" s="82"/>
+      <c r="BV4" s="87"/>
+      <c r="BW4" s="86">
         <f t="shared" ref="BW4" si="8">BW5</f>
         <v>45817</v>
       </c>
-      <c r="BX4" s="70"/>
-      <c r="BY4" s="70"/>
-      <c r="BZ4" s="70"/>
-      <c r="CA4" s="70"/>
-      <c r="CB4" s="70"/>
-      <c r="CC4" s="71"/>
-      <c r="CD4" s="69">
+      <c r="BX4" s="82"/>
+      <c r="BY4" s="82"/>
+      <c r="BZ4" s="82"/>
+      <c r="CA4" s="82"/>
+      <c r="CB4" s="82"/>
+      <c r="CC4" s="87"/>
+      <c r="CD4" s="86">
         <f t="shared" ref="CD4" si="9">CD5</f>
         <v>45824</v>
       </c>
-      <c r="CE4" s="70"/>
-      <c r="CF4" s="70"/>
-      <c r="CG4" s="70"/>
-      <c r="CH4" s="70"/>
-      <c r="CI4" s="70"/>
-      <c r="CJ4" s="71"/>
-      <c r="CK4" s="69">
+      <c r="CE4" s="82"/>
+      <c r="CF4" s="82"/>
+      <c r="CG4" s="82"/>
+      <c r="CH4" s="82"/>
+      <c r="CI4" s="82"/>
+      <c r="CJ4" s="87"/>
+      <c r="CK4" s="86">
         <f t="shared" ref="CK4" si="10">CK5</f>
         <v>45831</v>
       </c>
-      <c r="CL4" s="70"/>
-      <c r="CM4" s="70"/>
-      <c r="CN4" s="70"/>
-      <c r="CO4" s="70"/>
-      <c r="CP4" s="70"/>
-      <c r="CQ4" s="71"/>
-      <c r="CR4" s="69">
+      <c r="CL4" s="82"/>
+      <c r="CM4" s="82"/>
+      <c r="CN4" s="82"/>
+      <c r="CO4" s="82"/>
+      <c r="CP4" s="82"/>
+      <c r="CQ4" s="87"/>
+      <c r="CR4" s="86">
         <f t="shared" ref="CR4" si="11">CR5</f>
         <v>45838</v>
       </c>
-      <c r="CS4" s="70"/>
-      <c r="CT4" s="70"/>
-      <c r="CU4" s="70"/>
-      <c r="CV4" s="70"/>
-      <c r="CW4" s="70"/>
-      <c r="CX4" s="71"/>
+      <c r="CS4" s="82"/>
+      <c r="CT4" s="82"/>
+      <c r="CU4" s="82"/>
+      <c r="CV4" s="82"/>
+      <c r="CW4" s="82"/>
+      <c r="CX4" s="87"/>
     </row>
     <row r="5" spans="1:102" s="20" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A5" s="17" t="s">
@@ -1563,10 +1556,10 @@
       <c r="C5" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="73">
+      <c r="D5" s="84">
         <v>45754</v>
       </c>
-      <c r="E5" s="73"/>
+      <c r="E5" s="84"/>
       <c r="F5" s="44"/>
       <c r="G5" s="29"/>
       <c r="H5" s="43"/>
@@ -2832,7 +2825,7 @@
       <c r="H11" s="54">
         <v>45761</v>
       </c>
-      <c r="I11" s="75">
+      <c r="I11" s="69">
         <v>12</v>
       </c>
       <c r="J11" s="22"/>
@@ -2954,7 +2947,7 @@
       <c r="H12" s="54">
         <v>45777</v>
       </c>
-      <c r="I12" s="76">
+      <c r="I12" s="70">
         <v>4</v>
       </c>
       <c r="J12" s="22"/>
@@ -3076,7 +3069,7 @@
       <c r="H13" s="54">
         <v>45782</v>
       </c>
-      <c r="I13" s="77">
+      <c r="I13" s="71">
         <v>2</v>
       </c>
       <c r="J13" s="22"/>
@@ -3786,10 +3779,10 @@
       <c r="F19" s="51">
         <v>2</v>
       </c>
-      <c r="G19" s="78">
+      <c r="G19" s="72">
         <v>45761</v>
       </c>
-      <c r="H19" s="78">
+      <c r="H19" s="72">
         <v>45768</v>
       </c>
       <c r="I19" s="55">
@@ -3914,7 +3907,7 @@
       <c r="H20" s="54">
         <v>45792</v>
       </c>
-      <c r="I20" s="75">
+      <c r="I20" s="69">
         <v>1</v>
       </c>
       <c r="J20" s="22"/>
@@ -4158,7 +4151,7 @@
       <c r="H22" s="54">
         <v>45792</v>
       </c>
-      <c r="I22" s="75">
+      <c r="I22" s="69">
         <v>0.5</v>
       </c>
       <c r="J22" s="22"/>
@@ -4402,7 +4395,7 @@
       <c r="H24" s="54">
         <v>45817</v>
       </c>
-      <c r="I24" s="75">
+      <c r="I24" s="69">
         <v>1</v>
       </c>
       <c r="J24" s="22"/>
@@ -4524,7 +4517,7 @@
       <c r="H25" s="54">
         <v>45820</v>
       </c>
-      <c r="I25" s="75">
+      <c r="I25" s="69">
         <v>1</v>
       </c>
       <c r="J25" s="22"/>
@@ -4646,7 +4639,7 @@
       <c r="H26" s="54">
         <v>45831</v>
       </c>
-      <c r="I26" s="75">
+      <c r="I26" s="69">
         <v>5</v>
       </c>
       <c r="J26" s="22"/>
@@ -4868,13 +4861,13 @@
       <c r="F28" s="51">
         <v>4</v>
       </c>
-      <c r="G28" s="78">
+      <c r="G28" s="72">
         <v>45772</v>
       </c>
-      <c r="H28" s="78">
+      <c r="H28" s="72">
         <v>45772</v>
       </c>
-      <c r="I28" s="77">
+      <c r="I28" s="71">
         <v>3</v>
       </c>
       <c r="J28" s="22"/>
@@ -4990,13 +4983,13 @@
       <c r="F29" s="51">
         <v>4</v>
       </c>
-      <c r="G29" s="78">
+      <c r="G29" s="72">
         <v>45761</v>
       </c>
-      <c r="H29" s="78">
+      <c r="H29" s="72">
         <v>45768</v>
       </c>
-      <c r="I29" s="77">
+      <c r="I29" s="71">
         <v>3</v>
       </c>
       <c r="J29" s="22"/>
@@ -5240,7 +5233,7 @@
       <c r="H31" s="54">
         <v>45796</v>
       </c>
-      <c r="I31" s="77">
+      <c r="I31" s="71">
         <v>2</v>
       </c>
       <c r="J31" s="22"/>
@@ -5362,7 +5355,7 @@
       <c r="H32" s="54">
         <v>45803</v>
       </c>
-      <c r="I32" s="77">
+      <c r="I32" s="71">
         <v>3</v>
       </c>
       <c r="J32" s="22"/>
@@ -5728,7 +5721,7 @@
       <c r="H35" s="54">
         <v>45820</v>
       </c>
-      <c r="I35" s="77">
+      <c r="I35" s="71">
         <v>1</v>
       </c>
       <c r="J35" s="22"/>
@@ -5972,7 +5965,7 @@
       <c r="H37" s="54">
         <v>45838</v>
       </c>
-      <c r="I37" s="77">
+      <c r="I37" s="71">
         <v>8</v>
       </c>
       <c r="J37" s="22"/>
@@ -6319,7 +6312,7 @@
       <c r="G40" s="54">
         <v>45824</v>
       </c>
-      <c r="H40" s="78">
+      <c r="H40" s="72">
         <v>45834</v>
       </c>
       <c r="I40" s="56">
@@ -6438,7 +6431,7 @@
       <c r="G41" s="54">
         <v>45824</v>
       </c>
-      <c r="H41" s="78">
+      <c r="H41" s="72">
         <v>45834</v>
       </c>
       <c r="I41" s="55">
@@ -6553,108 +6546,15 @@
       <c r="F42" s="51">
         <v>8</v>
       </c>
-      <c r="G42" s="79">
+      <c r="G42" s="73">
         <v>45838</v>
       </c>
-      <c r="H42" s="79">
+      <c r="H42" s="73">
         <v>46130</v>
       </c>
       <c r="I42" s="56">
-        <v>90</v>
-      </c>
-      <c r="J42" s="80"/>
-      <c r="K42" s="82"/>
-      <c r="L42" s="82"/>
-      <c r="M42" s="82"/>
-      <c r="N42" s="82"/>
-      <c r="O42" s="82"/>
-      <c r="P42" s="82"/>
-      <c r="Q42" s="82"/>
-      <c r="R42" s="82"/>
-      <c r="S42" s="82"/>
-      <c r="T42" s="82"/>
-      <c r="U42" s="82"/>
-      <c r="V42" s="82"/>
-      <c r="W42" s="82"/>
-      <c r="X42" s="82"/>
-      <c r="Y42" s="82"/>
-      <c r="Z42" s="82"/>
-      <c r="AA42" s="82"/>
-      <c r="AB42" s="82"/>
-      <c r="AC42" s="82"/>
-      <c r="AD42" s="82"/>
-      <c r="AE42" s="82"/>
-      <c r="AF42" s="82"/>
-      <c r="AG42" s="82"/>
-      <c r="AH42" s="82"/>
-      <c r="AI42" s="82"/>
-      <c r="AJ42" s="82"/>
-      <c r="AK42" s="82"/>
-      <c r="AL42" s="82"/>
-      <c r="AM42" s="82"/>
-      <c r="AN42" s="82"/>
-      <c r="AO42" s="82"/>
-      <c r="AP42" s="82"/>
-      <c r="AQ42" s="82"/>
-      <c r="AR42" s="82"/>
-      <c r="AS42" s="82"/>
-      <c r="AT42" s="82"/>
-      <c r="AU42" s="82"/>
-      <c r="AV42" s="82"/>
-      <c r="AW42" s="82"/>
-      <c r="AX42" s="82"/>
-      <c r="AY42" s="82"/>
-      <c r="AZ42" s="82"/>
-      <c r="BA42" s="82"/>
-      <c r="BB42" s="82"/>
-      <c r="BC42" s="82"/>
-      <c r="BD42" s="82"/>
-      <c r="BE42" s="82"/>
-      <c r="BF42" s="82"/>
-      <c r="BG42" s="82"/>
-      <c r="BH42" s="82"/>
-      <c r="BI42" s="82"/>
-      <c r="BJ42" s="82"/>
-      <c r="BK42" s="82"/>
-      <c r="BL42" s="82"/>
-      <c r="BM42" s="82"/>
-      <c r="BN42" s="82"/>
-      <c r="BO42" s="82"/>
-      <c r="BP42" s="82"/>
-      <c r="BQ42" s="82"/>
-      <c r="BR42" s="82"/>
-      <c r="BS42" s="82"/>
-      <c r="BT42" s="82"/>
-      <c r="BU42" s="82"/>
-      <c r="BV42" s="82"/>
-      <c r="BW42" s="82"/>
-      <c r="BX42" s="82"/>
-      <c r="BY42" s="82"/>
-      <c r="BZ42" s="82"/>
-      <c r="CA42" s="82"/>
-      <c r="CB42" s="82"/>
-      <c r="CC42" s="82"/>
-      <c r="CD42" s="82"/>
-      <c r="CE42" s="82"/>
-      <c r="CF42" s="82"/>
-      <c r="CG42" s="82"/>
-      <c r="CH42" s="82"/>
-      <c r="CI42" s="82"/>
-      <c r="CJ42" s="82"/>
-      <c r="CK42" s="82"/>
-      <c r="CL42" s="82"/>
-      <c r="CM42" s="82"/>
-      <c r="CN42" s="82"/>
-      <c r="CO42" s="82"/>
-      <c r="CP42" s="82"/>
-      <c r="CQ42" s="82"/>
-      <c r="CR42" s="82"/>
-      <c r="CS42" s="82"/>
-      <c r="CT42" s="82"/>
-      <c r="CU42" s="82"/>
-      <c r="CV42" s="82"/>
-      <c r="CW42" s="82"/>
-      <c r="CX42" s="82"/>
+        <v>200</v>
+      </c>
     </row>
     <row r="43" spans="1:102" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A43" s="26"/>
@@ -6710,33 +6610,40 @@
     </row>
     <row r="49" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="50" spans="2:4" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B50" s="83" t="s">
+      <c r="B50" s="78" t="s">
         <v>59</v>
       </c>
-      <c r="C50" s="84"/>
-      <c r="D50" s="85">
+      <c r="C50" s="79"/>
+      <c r="D50" s="74">
         <f>SUM(F7:F42)</f>
         <v>180</v>
       </c>
     </row>
     <row r="51" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B51" s="86"/>
-      <c r="C51" s="81"/>
-      <c r="D51" s="87"/>
+      <c r="B51" s="75"/>
+      <c r="D51" s="76"/>
     </row>
     <row r="52" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B52" s="88" t="s">
+      <c r="B52" s="80" t="s">
         <v>60</v>
       </c>
-      <c r="C52" s="89"/>
-      <c r="D52" s="90">
+      <c r="C52" s="81"/>
+      <c r="D52" s="77">
         <f>SUM(I8:I42)</f>
-        <v>251.5</v>
+        <v>361.5</v>
       </c>
     </row>
     <row r="53" spans="2:4" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="CK4:CQ4"/>
+    <mergeCell ref="CR4:CX4"/>
+    <mergeCell ref="AU4:BA4"/>
+    <mergeCell ref="BB4:BH4"/>
+    <mergeCell ref="BI4:BO4"/>
+    <mergeCell ref="BP4:BV4"/>
+    <mergeCell ref="BW4:CC4"/>
+    <mergeCell ref="CD4:CJ4"/>
     <mergeCell ref="B50:C50"/>
     <mergeCell ref="B52:C52"/>
     <mergeCell ref="AN4:AT4"/>
@@ -6746,14 +6653,6 @@
     <mergeCell ref="S4:Y4"/>
     <mergeCell ref="Z4:AF4"/>
     <mergeCell ref="AG4:AM4"/>
-    <mergeCell ref="CK4:CQ4"/>
-    <mergeCell ref="CR4:CX4"/>
-    <mergeCell ref="AU4:BA4"/>
-    <mergeCell ref="BB4:BH4"/>
-    <mergeCell ref="BI4:BO4"/>
-    <mergeCell ref="BP4:BV4"/>
-    <mergeCell ref="BW4:CC4"/>
-    <mergeCell ref="CD4:CJ4"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="C48:C49 D44:D47 C51 C53:C1048576 C7:C43">

</xml_diff>